<commit_message>
feat(m3): unidades organizativas con vigencia, dimensiones por tenant y snapshots en el worker
</commit_message>
<xml_diff>
--- a/apps/cliente/public/examples/file_absenteeism.xlsx
+++ b/apps/cliente/public/examples/file_absenteeism.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="38">
   <si>
     <t>employee_code</t>
   </si>
@@ -67,6 +67,9 @@
     <t>2026-09-11</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>EMP002</t>
   </si>
   <si>
@@ -80,6 +83,48 @@
   </si>
   <si>
     <t>closed</t>
+  </si>
+  <si>
+    <t>EMP004</t>
+  </si>
+  <si>
+    <t>2026-09-08</t>
+  </si>
+  <si>
+    <t>2026-09-09</t>
+  </si>
+  <si>
+    <t>EMP005</t>
+  </si>
+  <si>
+    <t>EMP006</t>
+  </si>
+  <si>
+    <t>EMP007</t>
+  </si>
+  <si>
+    <t>2026-09-12</t>
+  </si>
+  <si>
+    <t>EMP008</t>
+  </si>
+  <si>
+    <t>2026-09-13</t>
+  </si>
+  <si>
+    <t>EMP009</t>
+  </si>
+  <si>
+    <t>2026-09-14</t>
+  </si>
+  <si>
+    <t>EMP010</t>
+  </si>
+  <si>
+    <t>EMP011</t>
+  </si>
+  <si>
+    <t>2026-09-16</t>
   </si>
 </sst>
 </file>
@@ -98,17 +143,12 @@
       <b/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE2E8F0"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -125,7 +165,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -465,15 +505,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="7" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="7" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -559,19 +598,22 @@
       <c r="H3" t="s">
         <v>12</v>
       </c>
+      <c r="I3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E4">
         <v>5</v>
@@ -583,7 +625,242 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="I4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>16</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>16</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>16</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>16</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <v>16</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10">
+        <v>16</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>23</v>
+      </c>
+      <c r="I10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11">
+        <v>16</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+      <c r="F12">
+        <v>16</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>